<commit_message>
add PDF Project Planning and UX Artefacts + update project task list
</commit_message>
<xml_diff>
--- a/docs/project-task-list.xlsx
+++ b/docs/project-task-list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D00283071\Desktop\2 YEAR\Server-side Development\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC5B306-2066-45D2-9ECD-8B3BA61333E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{711639AA-FCD9-46AF-90CB-5A751C329EC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
-  <si>
-    <t>Planning / UX tasks</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Project Concept and Problem Statement</t>
   </si>
@@ -91,6 +88,45 @@
   </si>
   <si>
     <t>In progress</t>
+  </si>
+  <si>
+    <t>STAGE-1 / Planning / UX tasks</t>
+  </si>
+  <si>
+    <t>STAGE-2 /</t>
+  </si>
+  <si>
+    <t>Create database and migrations</t>
+  </si>
+  <si>
+    <t>Implement authentication</t>
+  </si>
+  <si>
+    <t>Create Task model</t>
+  </si>
+  <si>
+    <t>Implement CRUD for tasks</t>
+  </si>
+  <si>
+    <t>Create Blade views</t>
+  </si>
+  <si>
+    <t>Add client-side validation</t>
+  </si>
+  <si>
+    <t>Add server-side validation</t>
+  </si>
+  <si>
+    <t>Test application</t>
+  </si>
+  <si>
+    <t>WEEK 23.03-29.03</t>
+  </si>
+  <si>
+    <t>WEEK 30.03-05.04</t>
+  </si>
+  <si>
+    <t>Maryna Hordiienko/Aleksy Cieslak</t>
   </si>
 </sst>
 </file>
@@ -178,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -190,6 +226,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -472,33 +512,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" customWidth="1"/>
     <col min="3" max="3" width="34.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" customWidth="1"/>
+    <col min="7" max="7" width="21.5703125" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>19</v>
-      </c>
       <c r="C1" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="F1" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
       <c r="J1" s="4"/>
@@ -506,13 +555,13 @@
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -523,13 +572,13 @@
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -541,10 +590,10 @@
       <c r="A4" s="1"/>
       <c r="B4" s="5"/>
       <c r="C4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -565,7 +614,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -576,7 +625,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="1"/>
@@ -589,14 +638,14 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -606,9 +655,11 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D9" s="1"/>
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>33</v>
+      </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -617,10 +668,10 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -630,9 +681,11 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="1"/>
+        <v>3</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
@@ -641,10 +694,11 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+        <v>4</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -652,10 +706,14 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
@@ -663,10 +721,11 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
@@ -674,10 +733,12 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
+      <c r="E15" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -685,10 +746,12 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C16" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+      <c r="E16" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -704,7 +767,9 @@
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C18" s="1"/>
+      <c r="C18" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -721,6 +786,95 @@
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
     </row>
+    <row r="20" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C21" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C22" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C23" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+    </row>
+    <row r="24" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C24" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C25" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+    </row>
+    <row r="26" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C26" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+    </row>
+    <row r="27" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C27" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A7:B7"/>

</xml_diff>

<commit_message>
excel update update as you wish if needed
</commit_message>
<xml_diff>
--- a/docs/project-task-list.xlsx
+++ b/docs/project-task-list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\H\WebstormProjects\task-planner\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E9B2EA-6B2D-4BC6-BE3C-914B4DD247FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0012D4CD-3451-464F-89A9-3CE18A91E7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
   <si>
     <t>Project Concept and Problem Statement</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>Maryna Hordiienko/Aleksy Cieslak</t>
+  </si>
+  <si>
+    <t>WEEK 06.04-12.04</t>
+  </si>
+  <si>
+    <t>Visual Appearance / CSS</t>
   </si>
 </sst>
 </file>
@@ -174,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -210,11 +216,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -225,10 +244,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -246,6 +272,92 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1876424</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>42862</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9948FBD7-CC40-942B-9B84-C0EE1912759C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3143249" y="5376862"/>
+          <a:ext cx="2714626" cy="914400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>Aleksy Cieslak:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100"/>
+            <a:t>Going to look</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
+            <a:t> over the project again today and tomorrow. There are bugs I encountered but overall quite pleased!</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -511,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" customWidth="1"/>
@@ -521,7 +633,7 @@
     <col min="5" max="5" width="30.7109375" customWidth="1"/>
     <col min="6" max="6" width="18.5703125" customWidth="1"/>
     <col min="7" max="7" width="21.5703125" customWidth="1"/>
-    <col min="8" max="8" width="13.28515625" customWidth="1"/>
+    <col min="8" max="8" width="33.140625" customWidth="1"/>
     <col min="9" max="9" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -547,7 +659,9 @@
       <c r="G1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="H1" s="6"/>
+      <c r="H1" s="6" t="s">
+        <v>34</v>
+      </c>
       <c r="I1" s="6"/>
       <c r="J1" s="4"/>
     </row>
@@ -623,10 +737,10 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="8"/>
+      <c r="A7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="12"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -639,7 +753,7 @@
       <c r="A8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="9"/>
+      <c r="B8" s="10"/>
       <c r="C8" s="1" t="s">
         <v>0</v>
       </c>
@@ -793,94 +907,116 @@
       <c r="E20" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C21" s="1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
+      <c r="E21" s="8"/>
       <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C22" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D22" s="1"/>
-      <c r="E22" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-      <c r="G22" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C23" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="E23" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
+      <c r="G23" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
     <row r="24" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C24" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D24" s="1"/>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="3" t="s">
         <v>15</v>
       </c>
       <c r="F24" s="1"/>
-      <c r="G24" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
     </row>
     <row r="25" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C25" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="E25" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
+      <c r="G25" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
     </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C26" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
+      <c r="H26" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="I26" s="1"/>
     </row>
     <row r="27" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C27" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
+      <c r="H27" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="I27" s="1"/>
+    </row>
+    <row r="28" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -888,5 +1024,6 @@
     <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated excel planning sheet
</commit_message>
<xml_diff>
--- a/docs/project-task-list.xlsx
+++ b/docs/project-task-list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\H\WebstormProjects\task-planner\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0012D4CD-3451-464F-89A9-3CE18A91E7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF0BFB2-7684-4E27-9264-E6CB6EF446D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
   <si>
     <t>Project Concept and Problem Statement</t>
   </si>
@@ -245,16 +245,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -272,92 +272,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1876424</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>42862</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9948FBD7-CC40-942B-9B84-C0EE1912759C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3143249" y="5376862"/>
-          <a:ext cx="2714626" cy="914400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1100"/>
-            <a:t>Aleksy Cieslak:</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1100"/>
-            <a:t>Going to look</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1100" baseline="0"/>
-            <a:t> over the project again today and tomorrow. There are bugs I encountered but overall quite pleased!</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-GB" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -737,10 +651,10 @@
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="12"/>
+      <c r="A7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="10"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -750,10 +664,10 @@
       <c r="I7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="1" t="s">
         <v>0</v>
       </c>
@@ -935,7 +849,9 @@
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
+      <c r="H22" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="I22" s="1"/>
     </row>
     <row r="23" spans="3:9" x14ac:dyDescent="0.25">
@@ -1024,6 +940,5 @@
     <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
create home page with focus tips and YouTube recommendation
</commit_message>
<xml_diff>
--- a/docs/project-task-list.xlsx
+++ b/docs/project-task-list.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\H\WebstormProjects\task-planner\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D00283071\Desktop\2 YEAR\Server-side Development\task-planner\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AF0BFB2-7684-4E27-9264-E6CB6EF446D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A766641-D030-4227-92BE-DECF098B1964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="37">
   <si>
     <t>Project Concept and Problem Statement</t>
   </si>
@@ -133,6 +144,9 @@
   </si>
   <si>
     <t>Visual Appearance / CSS</t>
+  </si>
+  <si>
+    <t>Create Home Page</t>
   </si>
 </sst>
 </file>
@@ -537,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" customWidth="1"/>
@@ -925,14 +939,27 @@
     </row>
     <row r="28" spans="3:9" x14ac:dyDescent="0.25">
       <c r="C28" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
+      <c r="H28" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>